<commit_message>
added cklickable launcher for all suppliers
</commit_message>
<xml_diff>
--- a/Icon/Icon_MATERIAL_PRICES.xlsx
+++ b/Icon/Icon_MATERIAL_PRICES.xlsx
@@ -28,9 +28,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy hh:mm"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -652,11 +651,11 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>97697</t>
+          <t>97112</t>
         </is>
       </c>
       <c r="J2" s="7" t="n">
-        <v>46287.64670673136</v>
+        <v>46288.46725976127</v>
       </c>
     </row>
     <row r="3">
@@ -685,11 +684,11 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>98272</t>
+          <t>96690</t>
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>46287.64670719444</v>
+        <v>46288.46725933856</v>
       </c>
     </row>
     <row r="4">
@@ -727,11 +726,11 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>98272</t>
+          <t>97112</t>
         </is>
       </c>
       <c r="J4" s="7" t="n">
-        <v>46287.64670719427</v>
+        <v>46288.46725976208</v>
       </c>
     </row>
     <row r="5">
@@ -764,7 +763,7 @@
         </is>
       </c>
       <c r="J5" s="7" t="n">
-        <v>46287.64670544065</v>
+        <v>46288.46725933904</v>
       </c>
     </row>
     <row r="6">
@@ -789,24 +788,24 @@
         </is>
       </c>
       <c r="E6" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F6" t="n">
         <v>5.19</v>
       </c>
-      <c r="F6" t="n">
-        <v>5.2</v>
-      </c>
       <c r="G6" t="n">
-        <v>-0.01</v>
+        <v>0.01</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-0.001923076923076923</v>
+        <v>0.001926782273603083</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>98272</t>
+          <t>97112</t>
         </is>
       </c>
       <c r="J6" s="7" t="n">
-        <v>46287.64670719325</v>
+        <v>46288.46725976162</v>
       </c>
     </row>
     <row r="7">
@@ -835,11 +834,11 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>98272</t>
+          <t>96690</t>
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>46287.64670719461</v>
+        <v>46288.46725933925</v>
       </c>
     </row>
     <row r="8">
@@ -872,7 +871,7 @@
         </is>
       </c>
       <c r="J8" s="7" t="n">
-        <v>46287.64670580468</v>
+        <v>46288.46725976219</v>
       </c>
     </row>
     <row r="9">
@@ -905,7 +904,7 @@
         </is>
       </c>
       <c r="J9" s="7" t="n">
-        <v>46287.6467058048</v>
+        <v>46288.46725976231</v>
       </c>
     </row>
     <row r="10">
@@ -938,7 +937,7 @@
         </is>
       </c>
       <c r="J10" s="7" t="n">
-        <v>46287.64670628771</v>
+        <v>46287.64670628472</v>
       </c>
     </row>
     <row r="11">
@@ -971,7 +970,7 @@
         </is>
       </c>
       <c r="J11" s="7" t="n">
-        <v>46287.64670628866</v>
+        <v>46287.64670628472</v>
       </c>
     </row>
     <row r="12">
@@ -1004,7 +1003,7 @@
         </is>
       </c>
       <c r="J12" s="7" t="n">
-        <v>46287.64670628909</v>
+        <v>46287.64670628472</v>
       </c>
     </row>
     <row r="13">
@@ -1037,7 +1036,7 @@
         </is>
       </c>
       <c r="J13" s="7" t="n">
-        <v>46287.64670673185</v>
+        <v>46287.64670673611</v>
       </c>
     </row>
     <row r="14">
@@ -1070,7 +1069,7 @@
         </is>
       </c>
       <c r="J14" s="7" t="n">
-        <v>46287.64670719256</v>
+        <v>46287.6467071875</v>
       </c>
     </row>
     <row r="15">
@@ -1103,7 +1102,7 @@
         </is>
       </c>
       <c r="J15" s="7" t="n">
-        <v>46287.64670719391</v>
+        <v>46287.64670719908</v>
       </c>
     </row>
     <row r="16">
@@ -1136,7 +1135,7 @@
         </is>
       </c>
       <c r="J16" s="7" t="n">
-        <v>46287.64670719494</v>
+        <v>46287.64670719908</v>
       </c>
     </row>
     <row r="17">
@@ -1169,7 +1168,7 @@
         </is>
       </c>
       <c r="J17" s="7" t="n">
-        <v>46287.64670752685</v>
+        <v>46287.64670752315</v>
       </c>
     </row>
   </sheetData>
@@ -1385,7 +1384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2148,6 +2147,105 @@
       <c r="G24" t="inlineStr">
         <is>
           <t>98716</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>05/05/2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ICV2692</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>S125R 125MM Round 2M Duct</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>17.92</v>
+      </c>
+      <c r="F25" t="n">
+        <v>15.58</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>96236</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ICV2692</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>S125R 125MM Round 2M Duct</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>15.58</v>
+      </c>
+      <c r="F26" t="n">
+        <v>17.92</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>96690</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>15/06/2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ICV245WH</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>100mm Cowled exhaust hood with damper WHITE</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>5.19</v>
+      </c>
+      <c r="F27" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>97112</t>
         </is>
       </c>
     </row>

</xml_diff>